<commit_message>
Large update in NCP and WasteCGE
</commit_message>
<xml_diff>
--- a/projects/WasteCGE/data/wasteDataFull.xlsx
+++ b/projects/WasteCGE/data/wasteDataFull.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxj477\Documents\GitHub\CGE_Generator\projects\WasteCGE\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2287A81E-B1E9-4230-8BBF-3F381607CD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282CABD7-7A85-4151-AF4E-0FA9917193BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="qd" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4298" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4300" uniqueCount="145">
   <si>
     <t>i</t>
   </si>
@@ -443,9 +443,6 @@
     <t>750000</t>
   </si>
   <si>
-    <t>rr</t>
-  </si>
-  <si>
     <t>we</t>
   </si>
   <si>
@@ -456,6 +453,15 @@
   </si>
   <si>
     <t>qWTE</t>
+  </si>
+  <si>
+    <t>A/R</t>
+  </si>
+  <si>
+    <t>dA/dR</t>
+  </si>
+  <si>
+    <t>R/W</t>
   </si>
 </sst>
 </file>
@@ -19425,47 +19431,77 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38143890-18C5-435B-B6D2-E0D473A90867}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="C1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0.78100000000000003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.80356000000000005</v>
+      </c>
+      <c r="C2">
+        <v>0.23996000000000001</v>
+      </c>
+      <c r="D2">
+        <v>0.969719</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
       <c r="B3">
-        <v>0.81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.80979000000000001</v>
+      </c>
+      <c r="C3">
+        <v>0.26577000000000001</v>
+      </c>
+      <c r="D3">
+        <v>0.99876600000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>55</v>
       </c>
       <c r="B4">
-        <v>0.26600000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.2666</v>
+      </c>
+      <c r="C4">
+        <v>1.4659999999999999E-2</v>
+      </c>
+      <c r="D4">
+        <v>0.93585700000000005</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>124</v>
       </c>
       <c r="B5">
-        <v>0.39200000000000002</v>
+        <v>0.46975</v>
+      </c>
+      <c r="C5">
+        <v>0.42903000000000002</v>
+      </c>
+      <c r="D5">
+        <v>0.26849699999999999</v>
       </c>
     </row>
   </sheetData>
@@ -19483,7 +19519,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -19541,7 +19577,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -19596,10 +19632,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" t="s">
         <v>141</v>
-      </c>
-      <c r="B1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>